<commit_message>
Update WeChat export: add 交易对方 column, remove 收款嫌疑账户
Co-authored-by: zhangliminabc <zhangliminabc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/微信支出记录表.xlsx
+++ b/微信支出记录表.xlsx
@@ -449,7 +449,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -461,9 +461,9 @@
           <t>被害人账户</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>收款嫌疑账户</t>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>交易对方</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -488,9 +488,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>10122606300300099756</t>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>老公🈲️⛔️姑奶奶</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -513,9 +513,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290331850759311</t>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>惜缘</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -538,9 +538,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290535003877356</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>火焰</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -563,9 +563,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290638778631642</t>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>TeL她的猫 TeL</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -588,9 +588,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290532876656891</t>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>TeL她的猫 TeL</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -613,9 +613,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290738748719105</t>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>南橘.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -638,11 +638,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290036239132427</t>
-        </is>
-      </c>
+      <c r="B8" s="4" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>53010003158196202606290261123505</t>
@@ -663,11 +659,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290037698260035</t>
-        </is>
-      </c>
+      <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
           <t>53010003280045202606290148190649</t>
@@ -688,11 +680,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290031258407265</t>
-        </is>
-      </c>
+      <c r="B10" s="4" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
           <t>53010003151035202606293245704329</t>
@@ -713,11 +701,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>10000500012026062900635283746852</t>
-        </is>
-      </c>
+      <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>53010003287097202606293212079344</t>
@@ -738,11 +722,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290337731082289</t>
-        </is>
-      </c>
+      <c r="B12" s="4" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>53010003266201202606292388317439</t>
@@ -763,11 +743,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290732760216074</t>
-        </is>
-      </c>
+      <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>53010003167227202606293649138649</t>
@@ -788,11 +764,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290632765862824</t>
-        </is>
-      </c>
+      <c r="B14" s="4" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>53010003277191202606292639783812</t>
@@ -813,9 +785,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290234876838821</t>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -838,9 +810,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290336012808241</t>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -863,11 +835,7 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290030020603876</t>
-        </is>
-      </c>
+      <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>53010003261019202606290101559530</t>
@@ -888,9 +856,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290638220346013</t>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -913,9 +881,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290536808116403</t>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -938,9 +906,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290733261908164</t>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -963,9 +931,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290531266420735</t>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -988,9 +956,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290035202731226</t>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1013,9 +981,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290239986577221</t>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1038,9 +1006,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290431532808626</t>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1063,9 +1031,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290237937677679</t>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1088,9 +1056,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290238995890280</t>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1113,9 +1081,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290436794371230</t>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1138,9 +1106,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290234816235181</t>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1163,9 +1131,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290233961971769</t>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1188,9 +1156,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290238676856604</t>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1213,9 +1181,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290433980830744</t>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1238,9 +1206,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290733784175792</t>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1263,9 +1231,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290036651615379</t>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1288,9 +1256,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290237800957074</t>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1313,9 +1281,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290234939902128</t>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1338,9 +1306,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290132621224994</t>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1363,9 +1331,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290038962169677</t>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -1388,9 +1356,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290238969795011</t>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1413,9 +1381,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290337496408406</t>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -1438,9 +1406,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290136553000692</t>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1463,9 +1431,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290131985749252</t>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1488,9 +1456,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290336441046417</t>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1513,9 +1481,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290331014943441</t>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -1538,9 +1506,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290234710181160</t>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -1563,9 +1531,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290436829069841</t>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -1588,9 +1556,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290734806349215</t>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -1613,9 +1581,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290330096106914</t>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1638,9 +1606,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290737887719185</t>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1663,9 +1631,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290537490129602</t>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -1688,9 +1656,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290230078874009</t>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -1713,9 +1681,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290735498551346</t>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -1738,9 +1706,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290432199839450</t>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -1763,9 +1731,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290632647081046</t>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -1788,9 +1756,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290232660482733</t>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -1813,9 +1781,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290437623395376</t>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -1838,9 +1806,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290737968187452</t>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -1863,9 +1831,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290639632700221</t>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -1888,9 +1856,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290634455423320</t>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -1913,9 +1881,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290131834902861</t>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -1938,9 +1906,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290732056456988</t>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -1963,9 +1931,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290136948489268</t>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -1988,9 +1956,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290138226407298</t>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2013,9 +1981,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290434325033713</t>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2038,9 +2006,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290338996181030</t>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -2063,9 +2031,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290130143881290</t>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -2088,9 +2056,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290739389266976</t>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -2113,9 +2081,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290232288080904</t>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -2138,9 +2106,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290336579127914</t>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2163,9 +2131,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290531591022320</t>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -2188,9 +2156,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290438208787559</t>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -2213,9 +2181,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290339391647912</t>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -2238,9 +2206,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290436832526725</t>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -2263,9 +2231,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290138944090239</t>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -2288,9 +2256,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290334221468091</t>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -2313,9 +2281,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290030360899358</t>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -2338,9 +2306,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290235533854595</t>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -2363,9 +2331,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290338500963869</t>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -2388,9 +2356,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290537057864476</t>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -2413,9 +2381,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290634797513581</t>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -2438,9 +2406,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290735077737919</t>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -2463,9 +2431,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290133344223295</t>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -2488,9 +2456,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290237283171241</t>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -2513,9 +2481,9 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>1000050001202606290236705799719</t>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add 62 more WeChat expenditure records from 5 new images
Co-authored-by: zhangliminabc <zhangliminabc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/微信支出记录表.xlsx
+++ b/微信支出记录表.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2500,14 +2500,1564 @@
         <v>190</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>53010003253173202606291394855761</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:06:34</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
     <row r="85">
-      <c r="D85" s="5" t="inlineStr">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>53010003161140202606290452260031</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:06:25</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>53010003278108202606290016388056</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:06:15</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>53010003154220202606291912979631</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:06:05</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>53010003163019202606290623798372</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:05:55</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>53010003249203202606290542667249</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:04:57</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>53010003270065202606291572033644</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:04:46</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>53010003165160202606290178428499</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:04:36</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>53010003287035202606293653765643</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:04:26</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>53010003275078202606293566877532</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:04:14</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>53010003163141202606293058374235</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:04:05</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>53010003247059202606291603089336</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:03:55</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>53010003272012202606290137162540</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:03:45</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>53010003274228202606294259225011</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:03:31</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>53010003150253202606294276177985</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:03:21</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>53010003256007202606291178261054</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:03:10</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>53010003150086202606292817497088</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:02:58</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>53010003150163202606290906867345</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:02:48</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>53010003262010202606290664904950</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:02:38</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>53010003274206202606293328179654</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:02:28</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>53010003279223202606290433196161</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:02:18</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>53010003247006202606291869721971</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:02:08</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>53010003167046202606292044534585</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:01:58</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>53010003155222202606293214583527</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:01:48</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>53010003283179202606292426620425</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:01:38</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>53010003275104202606291147831507</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:01:24</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>53010003267125202606291131277446</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:01:13</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>53010003251192202606290933286963</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:01:01</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>53010003249172202606290057305220</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:00:14</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>53010003145016202606291109155408</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 16:00:02</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>53010003157116202606292776194880</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:59:50</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>53010003279069202606292346066896</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:59:38</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>53010003148242202606293881337035</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:59:26</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>53010003253211202606292307629930</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:59:14</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>53010003158193202606293242758790</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:59:04</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>53010003263011202606293868792043</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:58:51</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>53010003149105202606291522923483</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:58:39</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>53010003261104202606291821494577</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:58:26</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>53010003282161202606293517093759</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:58:14</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>53010003268105202606293361673274</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:58:02</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>53010003290086202606291153902679</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:57:50</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>53010003166000202606291764940034</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:57:38</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>53010003271204202606290181552837</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:57:25</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>53010003282035202606290590911578</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:57:15</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>53010003284072202606291964060749</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:56:57</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>53010003273107202606293076874598</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:56:47</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>53010003144104202606294024076281</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:56:37</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>53010003282126202606290211371154</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:56:27</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>53010003280188202606292664243214</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:56:17</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>53010003287162202606290064803261</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:56:07</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>53010003165248202606293511058812</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:55:57</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>53010003268115202606292201325098</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:55:47</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>53010003256037202606291433061585</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:55:37</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>53010003294048202606291918943726</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:55:27</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>53010003151169202606292554837411</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:55:16</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>53010003156164202606293673134992</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:55:04</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>53010003285227202606291087429253</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:54:52</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>53010003166222202606290873937400</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:54:41</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>53010003251079202606292549047594</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:54:28</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>530100032552202606291979520460</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:54:06</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>53010003161222202606290281335611</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:53:54</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>53010003264194202606293887561808</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:53:42</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="D147" s="5" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="E85" s="5" t="n">
-        <v>50421.79</v>
+      <c r="E147" s="5" t="n">
+        <v>61351.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 18 expenditure records, exclude 交易对方为惜缘
Co-authored-by: zhangliminabc <zhangliminabc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/微信支出记录表.xlsx
+++ b/微信支出记录表.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E147"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -515,21 +515,21 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>惜缘</t>
+          <t>火焰</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>53010003283108202606291902162066</t>
+          <t>53010003147049202606290702526477</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 18:14:48</t>
+          <t>2026-06-29 18:00:54</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>5000</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4">
@@ -540,21 +540,21 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>火焰</t>
+          <t>TeL她的猫 TeL</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>53010003147049202606290702526477</t>
+          <t>53010003284222202606290442370984</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 18:00:54</t>
+          <t>2026-06-29 17:59:44</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>150</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">
@@ -570,12 +570,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>53010003284222202606290442370984</t>
+          <t>53010003250008202606290091406333</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:59:44</t>
+          <t>2026-06-29 17:59:27</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
@@ -590,21 +590,21 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>TeL她的猫 TeL</t>
+          <t>南橘.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>53010003250008202606290091406333</t>
+          <t>53010003166199202606291335094798</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:59:27</t>
+          <t>2026-06-29 17:57:58</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>99</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7">
@@ -613,19 +613,15 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>南橘.</t>
-        </is>
-      </c>
+      <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>53010003166199202606291335094798</t>
+          <t>53010003158196202606290261123505</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:57:58</t>
+          <t>2026-06-29 17:48:29</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
@@ -641,16 +637,16 @@
       <c r="B8" s="4" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>53010003158196202606290261123505</t>
+          <t>53010003280045202606290148190649</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:48:29</t>
+          <t>2026-06-29 17:45:58</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9">
@@ -662,16 +658,16 @@
       <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>53010003280045202606290148190649</t>
+          <t>53010003151035202606293245704329</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:45:58</t>
+          <t>2026-06-29 17:40:24</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>130</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10">
@@ -683,12 +679,12 @@
       <c r="B10" s="4" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>53010003151035202606293245704329</t>
+          <t>53010003287097202606293212079344</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:40:24</t>
+          <t>2026-06-29 17:40:12</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
@@ -704,16 +700,16 @@
       <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>53010003287097202606293212079344</t>
+          <t>53010003266201202606292388317439</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:40:12</t>
+          <t>2026-06-29 17:33:02</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>99</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12">
@@ -725,16 +721,16 @@
       <c r="B12" s="4" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>53010003266201202606292388317439</t>
+          <t>53010003167227202606293649138649</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:33:02</t>
+          <t>2026-06-29 17:29:27</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>110</v>
+        <v>31326</v>
       </c>
     </row>
     <row r="13">
@@ -746,16 +742,16 @@
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>53010003167227202606293649138649</t>
+          <t>53010003277191202606292639783812</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 17:29:27</t>
+          <t>2026-06-29 16:23:57</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>31326</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
@@ -764,19 +760,23 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>53010003277191202606292639783812</t>
+          <t>53010003251026202606294290691031</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:23:57</t>
+          <t>2026-06-29 16:23:36</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>60</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15">
@@ -792,12 +792,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>53010003251026202606294290691031</t>
+          <t>53010003288138202606293332309515</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:23:36</t>
+          <t>2026-06-29 16:23:14</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
@@ -810,23 +810,19 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>KK</t>
-        </is>
-      </c>
+      <c r="B16" s="4" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>53010003288138202606293332309515</t>
+          <t>53010003261019202606290101559530</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:23:14</t>
+          <t>2026-06-29 16:19:29</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>190</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -835,19 +831,23 @@
           <t>18428341745</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>53010003261019202606290101559530</t>
+          <t>53010003290208202606292930295298</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:19:29</t>
+          <t>2026-06-29 16:19:05</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>100</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18">
@@ -863,12 +863,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>53010003290208202606292930295298</t>
+          <t>53010003156010202606293605378283</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:19:05</t>
+          <t>2026-06-29 16:18:56</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
@@ -888,12 +888,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>53010003156010202606293605378283</t>
+          <t>53010003163062202606293910451226</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:18:56</t>
+          <t>2026-06-29 16:18:46</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
@@ -913,12 +913,12 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>53010003163062202606293910451226</t>
+          <t>53010003286152202606293926991488</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:18:46</t>
+          <t>2026-06-29 16:18:34</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
@@ -938,12 +938,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>53010003286152202606293926991488</t>
+          <t>530100032500202606290834886070</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:18:34</t>
+          <t>2026-06-29 16:18:25</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
@@ -963,12 +963,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>530100032500202606290834886070</t>
+          <t>53010003251207202606290969954738</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:18:25</t>
+          <t>2026-06-29 16:17:52</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
@@ -988,12 +988,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>53010003251207202606290969954738</t>
+          <t>53010003147034202606290635363707</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:17:52</t>
+          <t>2026-06-29 16:17:42</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>53010003147034202606290635363707</t>
+          <t>53010003280211202606292992548991</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:17:42</t>
+          <t>2026-06-29 16:17:31</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>53010003280211202606292992548991</t>
+          <t>53010003154006202606290218396396</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:17:31</t>
+          <t>2026-06-29 16:17:22</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
@@ -1063,12 +1063,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>53010003154006202606290218396396</t>
+          <t>53010003165041202606290080001546</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:17:22</t>
+          <t>2026-06-29 16:17:09</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
@@ -1088,12 +1088,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>53010003165041202606290080001546</t>
+          <t>53010003250048202606290823638361</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:17:09</t>
+          <t>2026-06-29 16:16:53</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
@@ -1113,12 +1113,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>53010003250048202606290823638361</t>
+          <t>53010003155050202606292271304563</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:16:53</t>
+          <t>2026-06-29 16:16:40</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
@@ -1138,12 +1138,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>53010003155050202606292271304563</t>
+          <t>53010003272087202606291955780025</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:16:40</t>
+          <t>2026-06-29 16:16:31</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>53010003272087202606291955780025</t>
+          <t>53010003164122202606291791566327</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:16:31</t>
+          <t>2026-06-29 16:16:21</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>53010003164122202606291791566327</t>
+          <t>53010003167230202606291736125727</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:16:21</t>
+          <t>2026-06-29 16:16:09</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>53010003167230202606291736125727</t>
+          <t>53010003150194202606292877185148</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:16:09</t>
+          <t>2026-06-29 16:16:00</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
@@ -1238,12 +1238,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>53010003150194202606292877185148</t>
+          <t>53010003250113202606293002609244</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:16:00</t>
+          <t>2026-06-29 16:15:29</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -1263,12 +1263,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>53010003250113202606293002609244</t>
+          <t>53010003165067202606292486284326</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:15:29</t>
+          <t>2026-06-29 16:15:17</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>53010003165067202606292486284326</t>
+          <t>53010003265232202606293912699513</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:15:17</t>
+          <t>2026-06-29 16:15:08</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>53010003265232202606293912699513</t>
+          <t>53010003155199202606293965013652</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:15:08</t>
+          <t>2026-06-29 16:14:58</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
@@ -1338,12 +1338,12 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>53010003155199202606293965013652</t>
+          <t>53010003145183202606291926137236</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:14:58</t>
+          <t>2026-06-29 16:14:48</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>53010003145183202606291926137236</t>
+          <t>53010003155019202606293854465025</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:14:48</t>
+          <t>2026-06-29 16:14:37</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
@@ -1388,12 +1388,12 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>53010003155019202606293854465025</t>
+          <t>53010003252236202606294166650249</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:14:37</t>
+          <t>2026-06-29 16:14:27</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
@@ -1413,12 +1413,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>53010003252236202606294166650249</t>
+          <t>53010003255234202606293623420363</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:14:27</t>
+          <t>2026-06-29 16:14:17</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>53010003255234202606293623420363</t>
+          <t>53010003150097202606291103290735</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:14:17</t>
+          <t>2026-06-29 16:14:08</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
@@ -1463,12 +1463,12 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>53010003150097202606291103290735</t>
+          <t>53010003261148202606290364289111</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:14:08</t>
+          <t>2026-06-29 16:13:57</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
@@ -1488,12 +1488,12 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>53010003261148202606290364289111</t>
+          <t>53010003164056202606290230676653</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:13:57</t>
+          <t>2026-06-29 16:13:45</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
@@ -1513,12 +1513,12 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>53010003164056202606290230676653</t>
+          <t>53010003247115202606292564117715</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:13:45</t>
+          <t>2026-06-29 16:13:33</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>53010003247115202606292564117715</t>
+          <t>53010003285118202606290536592984</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:13:33</t>
+          <t>2026-06-29 16:13:23</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>53010003285118202606290536592984</t>
+          <t>53010003153195202606291133116508</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:13:23</t>
+          <t>2026-06-29 16:13:13</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>53010003153195202606291133116508</t>
+          <t>53010003154042202606293314335540</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:13:13</t>
+          <t>2026-06-29 16:13:03</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
@@ -1613,12 +1613,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>53010003154042202606293314335540</t>
+          <t>53010003247142202606291921570396</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:13:03</t>
+          <t>2026-06-29 16:12:53</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>53010003247142202606291921570396</t>
+          <t>53010003145189202606294133593738</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:12:53</t>
+          <t>2026-06-29 16:12:43</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>53010003145189202606294133593738</t>
+          <t>53010003153192202606290675383273</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:12:43</t>
+          <t>2026-06-29 16:12:33</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
@@ -1688,12 +1688,12 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>53010003153192202606290675383273</t>
+          <t>53010003270082202606291946758529</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:12:33</t>
+          <t>2026-06-29 16:12:23</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
@@ -1713,12 +1713,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>53010003270082202606291946758529</t>
+          <t>53010003250118202606290300197190</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:12:23</t>
+          <t>2026-06-29 16:12:13</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
@@ -1738,12 +1738,12 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>53010003250118202606290300197190</t>
+          <t>53010003295021202606291161206767</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:12:13</t>
+          <t>2026-06-29 16:12:03</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
@@ -1763,12 +1763,12 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>53010003295021202606291161206767</t>
+          <t>53010003251165202606290200521443</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:12:03</t>
+          <t>2026-06-29 16:11:52</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
@@ -1788,12 +1788,12 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>53010003251165202606290200521443</t>
+          <t>53010003156017202606292896014649</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:11:52</t>
+          <t>2026-06-29 16:11:42</t>
         </is>
       </c>
       <c r="E55" s="4" t="n">
@@ -1813,12 +1813,12 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>53010003156017202606292896014649</t>
+          <t>53010003275110202606290455136171</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:11:42</t>
+          <t>2026-06-29 16:11:32</t>
         </is>
       </c>
       <c r="E56" s="4" t="n">
@@ -1838,12 +1838,12 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>53010003275110202606290455136171</t>
+          <t>53010003254038202606291392028278</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:11:32</t>
+          <t>2026-06-29 16:11:22</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>53010003254038202606291392028278</t>
+          <t>53010003254111202606292973146865</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:11:22</t>
+          <t>2026-06-29 16:11:12</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>53010003254111202606292973146865</t>
+          <t>53010003151130202606291893513573</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:11:12</t>
+          <t>2026-06-29 16:11:01</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>53010003151130202606291893513573</t>
+          <t>53010003280052202606293325133438</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:11:01</t>
+          <t>2026-06-29 16:10:46</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
@@ -1938,12 +1938,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>53010003280052202606293325133438</t>
+          <t>53010003253051202606293709070928</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:10:46</t>
+          <t>2026-06-29 16:10:36</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>53010003253051202606293709070928</t>
+          <t>53010003148217202606290063658993</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:10:36</t>
+          <t>2026-06-29 16:10:25</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
@@ -1988,12 +1988,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>53010003148217202606290063658993</t>
+          <t>53010003162206202606290899325347</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:10:25</t>
+          <t>2026-06-29 16:10:15</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
@@ -2013,12 +2013,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>53010003162206202606290899325347</t>
+          <t>53010003155024202606292502702256</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:10:15</t>
+          <t>2026-06-29 16:10:06</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
@@ -2038,12 +2038,12 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>53010003155024202606292502702256</t>
+          <t>53010003149193202606292196473713</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:10:06</t>
+          <t>2026-06-29 16:09:57</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>53010003149193202606292196473713</t>
+          <t>53010003282078202606291699878914</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:09:57</t>
+          <t>2026-06-29 16:09:47</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
@@ -2088,12 +2088,12 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>53010003282078202606291699878914</t>
+          <t>53010003276113202606292625403302</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:09:47</t>
+          <t>2026-06-29 16:09:25</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
@@ -2113,12 +2113,12 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>53010003276113202606292625403302</t>
+          <t>53010003161098202606292661281269</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:09:25</t>
+          <t>2026-06-29 16:09:15</t>
         </is>
       </c>
       <c r="E68" s="4" t="n">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>53010003161098202606292661281269</t>
+          <t>53010003266072202606290257942903</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:09:15</t>
+          <t>2026-06-29 16:09:05</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
@@ -2163,12 +2163,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>53010003266072202606290257942903</t>
+          <t>53010003282023202606290137022178</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:09:05</t>
+          <t>2026-06-29 16:08:55</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
@@ -2188,12 +2188,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>53010003282023202606290137022178</t>
+          <t>53010003249141202606293659969155</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:08:55</t>
+          <t>2026-06-29 16:08:46</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
@@ -2213,12 +2213,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>53010003249141202606293659969155</t>
+          <t>53010003150073202606293581685461</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:08:46</t>
+          <t>2026-06-29 16:08:35</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>53010003150073202606293581685461</t>
+          <t>53010003265251202606290262549501</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:08:35</t>
+          <t>2026-06-29 16:08:25</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
@@ -2263,12 +2263,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>53010003265251202606290262549501</t>
+          <t>53010003266240202606292062478496</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:08:25</t>
+          <t>2026-06-29 16:08:09</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
@@ -2288,12 +2288,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>53010003266240202606292062478496</t>
+          <t>53010003266130202606293184872186</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:08:09</t>
+          <t>2026-06-29 16:08:00</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>53010003266130202606293184872186</t>
+          <t>53010003156029202606293935097747</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:08:00</t>
+          <t>2026-06-29 16:07:48</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
@@ -2338,12 +2338,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>53010003156029202606293935097747</t>
+          <t>53010003155002202606292419168182</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:07:48</t>
+          <t>2026-06-29 16:07:38</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
@@ -2363,12 +2363,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>53010003155002202606292419168182</t>
+          <t>53010003287035202606292044470301</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:07:38</t>
+          <t>2026-06-29 16:07:27</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
@@ -2388,12 +2388,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>53010003287035202606292044470301</t>
+          <t>53010003262047202606291946383912</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:07:27</t>
+          <t>2026-06-29 16:07:18</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
@@ -2413,12 +2413,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>53010003262047202606291946383912</t>
+          <t>53010003272077202606291264893000</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:07:18</t>
+          <t>2026-06-29 16:07:08</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
@@ -2438,12 +2438,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>53010003272077202606291264893000</t>
+          <t>53010003285197202606291632429112</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:07:08</t>
+          <t>2026-06-29 16:06:53</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
@@ -2463,12 +2463,12 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>53010003285197202606291632429112</t>
+          <t>53010003282144202606290962509880</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:06:53</t>
+          <t>2026-06-29 16:06:43</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
@@ -2488,12 +2488,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>53010003282144202606290962509880</t>
+          <t>53010003253173202606291394855761</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:06:43</t>
+          <t>2026-06-29 16:06:34</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
@@ -2513,12 +2513,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>53010003253173202606291394855761</t>
+          <t>53010003161140202606290452260031</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:06:34</t>
+          <t>2026-06-29 16:06:25</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
@@ -2538,12 +2538,12 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>53010003161140202606290452260031</t>
+          <t>53010003278108202606290016388056</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:06:25</t>
+          <t>2026-06-29 16:06:15</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>53010003278108202606290016388056</t>
+          <t>53010003154220202606291912979631</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:06:15</t>
+          <t>2026-06-29 16:06:05</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
@@ -2588,12 +2588,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>53010003154220202606291912979631</t>
+          <t>53010003163019202606290623798372</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:06:05</t>
+          <t>2026-06-29 16:05:55</t>
         </is>
       </c>
       <c r="E87" s="4" t="n">
@@ -2613,12 +2613,12 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>53010003163019202606290623798372</t>
+          <t>53010003249203202606290542667249</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:05:55</t>
+          <t>2026-06-29 16:04:57</t>
         </is>
       </c>
       <c r="E88" s="4" t="n">
@@ -2638,12 +2638,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>53010003249203202606290542667249</t>
+          <t>53010003270065202606291572033644</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:04:57</t>
+          <t>2026-06-29 16:04:46</t>
         </is>
       </c>
       <c r="E89" s="4" t="n">
@@ -2663,12 +2663,12 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>53010003270065202606291572033644</t>
+          <t>53010003165160202606290178428499</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:04:46</t>
+          <t>2026-06-29 16:04:36</t>
         </is>
       </c>
       <c r="E90" s="4" t="n">
@@ -2688,12 +2688,12 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>53010003165160202606290178428499</t>
+          <t>53010003287035202606293653765643</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:04:36</t>
+          <t>2026-06-29 16:04:26</t>
         </is>
       </c>
       <c r="E91" s="4" t="n">
@@ -2713,12 +2713,12 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>53010003287035202606293653765643</t>
+          <t>53010003275078202606293566877532</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:04:26</t>
+          <t>2026-06-29 16:04:14</t>
         </is>
       </c>
       <c r="E92" s="4" t="n">
@@ -2738,12 +2738,12 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>53010003275078202606293566877532</t>
+          <t>53010003163141202606293058374235</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:04:14</t>
+          <t>2026-06-29 16:04:05</t>
         </is>
       </c>
       <c r="E93" s="4" t="n">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>53010003163141202606293058374235</t>
+          <t>53010003247059202606291603089336</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:04:05</t>
+          <t>2026-06-29 16:03:55</t>
         </is>
       </c>
       <c r="E94" s="4" t="n">
@@ -2788,12 +2788,12 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>53010003247059202606291603089336</t>
+          <t>53010003272012202606290137162540</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:03:55</t>
+          <t>2026-06-29 16:03:45</t>
         </is>
       </c>
       <c r="E95" s="4" t="n">
@@ -2813,12 +2813,12 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>53010003272012202606290137162540</t>
+          <t>53010003274228202606294259225011</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:03:45</t>
+          <t>2026-06-29 16:03:31</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>53010003274228202606294259225011</t>
+          <t>53010003150253202606294276177985</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:03:31</t>
+          <t>2026-06-29 16:03:21</t>
         </is>
       </c>
       <c r="E97" s="4" t="n">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>53010003150253202606294276177985</t>
+          <t>53010003256007202606291178261054</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:03:21</t>
+          <t>2026-06-29 16:03:10</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
@@ -2888,12 +2888,12 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>53010003256007202606291178261054</t>
+          <t>53010003150086202606292817497088</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:03:10</t>
+          <t>2026-06-29 16:02:58</t>
         </is>
       </c>
       <c r="E99" s="4" t="n">
@@ -2913,12 +2913,12 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>53010003150086202606292817497088</t>
+          <t>53010003150163202606290906867345</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:02:58</t>
+          <t>2026-06-29 16:02:48</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>53010003150163202606290906867345</t>
+          <t>53010003262010202606290664904950</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:02:48</t>
+          <t>2026-06-29 16:02:38</t>
         </is>
       </c>
       <c r="E101" s="4" t="n">
@@ -2963,12 +2963,12 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>53010003262010202606290664904950</t>
+          <t>53010003274206202606293328179654</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:02:38</t>
+          <t>2026-06-29 16:02:28</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
@@ -2988,12 +2988,12 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>53010003274206202606293328179654</t>
+          <t>53010003279223202606290433196161</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:02:28</t>
+          <t>2026-06-29 16:02:18</t>
         </is>
       </c>
       <c r="E103" s="4" t="n">
@@ -3013,12 +3013,12 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>53010003279223202606290433196161</t>
+          <t>53010003247006202606291869721971</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:02:18</t>
+          <t>2026-06-29 16:02:08</t>
         </is>
       </c>
       <c r="E104" s="4" t="n">
@@ -3038,12 +3038,12 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>53010003247006202606291869721971</t>
+          <t>53010003167046202606292044534585</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:02:08</t>
+          <t>2026-06-29 16:01:58</t>
         </is>
       </c>
       <c r="E105" s="4" t="n">
@@ -3063,12 +3063,12 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>53010003167046202606292044534585</t>
+          <t>53010003155222202606293214583527</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:01:58</t>
+          <t>2026-06-29 16:01:48</t>
         </is>
       </c>
       <c r="E106" s="4" t="n">
@@ -3088,12 +3088,12 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>53010003155222202606293214583527</t>
+          <t>53010003283179202606292426620425</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:01:48</t>
+          <t>2026-06-29 16:01:38</t>
         </is>
       </c>
       <c r="E107" s="4" t="n">
@@ -3113,12 +3113,12 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>53010003283179202606292426620425</t>
+          <t>53010003275104202606291147831507</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:01:38</t>
+          <t>2026-06-29 16:01:24</t>
         </is>
       </c>
       <c r="E108" s="4" t="n">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>53010003275104202606291147831507</t>
+          <t>53010003267125202606291131277446</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:01:24</t>
+          <t>2026-06-29 16:01:13</t>
         </is>
       </c>
       <c r="E109" s="4" t="n">
@@ -3163,12 +3163,12 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>53010003267125202606291131277446</t>
+          <t>53010003251192202606290933286963</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:01:13</t>
+          <t>2026-06-29 16:01:01</t>
         </is>
       </c>
       <c r="E110" s="4" t="n">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>53010003251192202606290933286963</t>
+          <t>53010003249172202606290057305220</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:01:01</t>
+          <t>2026-06-29 16:00:14</t>
         </is>
       </c>
       <c r="E111" s="4" t="n">
@@ -3213,12 +3213,12 @@
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>53010003249172202606290057305220</t>
+          <t>53010003145016202606291109155408</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:00:14</t>
+          <t>2026-06-29 16:00:02</t>
         </is>
       </c>
       <c r="E112" s="4" t="n">
@@ -3238,12 +3238,12 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>53010003145016202606291109155408</t>
+          <t>53010003157116202606292776194880</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 16:00:02</t>
+          <t>2026-06-29 15:59:50</t>
         </is>
       </c>
       <c r="E113" s="4" t="n">
@@ -3263,12 +3263,12 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>53010003157116202606292776194880</t>
+          <t>53010003279069202606292346066896</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:59:50</t>
+          <t>2026-06-29 15:59:38</t>
         </is>
       </c>
       <c r="E114" s="4" t="n">
@@ -3288,12 +3288,12 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>53010003279069202606292346066896</t>
+          <t>53010003148242202606293881337035</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:59:38</t>
+          <t>2026-06-29 15:59:26</t>
         </is>
       </c>
       <c r="E115" s="4" t="n">
@@ -3313,12 +3313,12 @@
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>53010003148242202606293881337035</t>
+          <t>53010003253211202606292307629930</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:59:26</t>
+          <t>2026-06-29 15:59:14</t>
         </is>
       </c>
       <c r="E116" s="4" t="n">
@@ -3338,16 +3338,16 @@
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>53010003253211202606292307629930</t>
+          <t>53010003158193202606293242758790</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:59:14</t>
+          <t>2026-06-29 15:59:04</t>
         </is>
       </c>
       <c r="E117" s="4" t="n">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="118">
@@ -3363,12 +3363,12 @@
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>53010003158193202606293242758790</t>
+          <t>53010003263011202606293868792043</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:59:04</t>
+          <t>2026-06-29 15:58:51</t>
         </is>
       </c>
       <c r="E118" s="4" t="n">
@@ -3388,12 +3388,12 @@
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>53010003263011202606293868792043</t>
+          <t>53010003149105202606291522923483</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:58:51</t>
+          <t>2026-06-29 15:58:39</t>
         </is>
       </c>
       <c r="E119" s="4" t="n">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>53010003149105202606291522923483</t>
+          <t>53010003261104202606291821494577</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:58:39</t>
+          <t>2026-06-29 15:58:26</t>
         </is>
       </c>
       <c r="E120" s="4" t="n">
@@ -3438,12 +3438,12 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>53010003261104202606291821494577</t>
+          <t>53010003282161202606293517093759</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:58:26</t>
+          <t>2026-06-29 15:58:14</t>
         </is>
       </c>
       <c r="E121" s="4" t="n">
@@ -3463,12 +3463,12 @@
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>53010003282161202606293517093759</t>
+          <t>53010003268105202606293361673274</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:58:14</t>
+          <t>2026-06-29 15:58:02</t>
         </is>
       </c>
       <c r="E122" s="4" t="n">
@@ -3488,12 +3488,12 @@
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>53010003268105202606293361673274</t>
+          <t>53010003290086202606291153902679</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:58:02</t>
+          <t>2026-06-29 15:57:50</t>
         </is>
       </c>
       <c r="E123" s="4" t="n">
@@ -3513,12 +3513,12 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>53010003290086202606291153902679</t>
+          <t>53010003166000202606291764940034</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:57:50</t>
+          <t>2026-06-29 15:57:38</t>
         </is>
       </c>
       <c r="E124" s="4" t="n">
@@ -3538,12 +3538,12 @@
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>53010003166000202606291764940034</t>
+          <t>53010003271204202606290181552837</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:57:38</t>
+          <t>2026-06-29 15:57:25</t>
         </is>
       </c>
       <c r="E125" s="4" t="n">
@@ -3563,16 +3563,16 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>53010003271204202606290181552837</t>
+          <t>53010003282035202606290590911578</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:57:25</t>
+          <t>2026-06-29 15:57:15</t>
         </is>
       </c>
       <c r="E126" s="4" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
     </row>
     <row r="127">
@@ -3588,12 +3588,12 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>53010003282035202606290590911578</t>
+          <t>53010003284072202606291964060749</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:57:15</t>
+          <t>2026-06-29 15:56:57</t>
         </is>
       </c>
       <c r="E127" s="4" t="n">
@@ -3613,12 +3613,12 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>53010003284072202606291964060749</t>
+          <t>53010003273107202606293076874598</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:56:57</t>
+          <t>2026-06-29 15:56:47</t>
         </is>
       </c>
       <c r="E128" s="4" t="n">
@@ -3638,12 +3638,12 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>53010003273107202606293076874598</t>
+          <t>53010003144104202606294024076281</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:56:47</t>
+          <t>2026-06-29 15:56:37</t>
         </is>
       </c>
       <c r="E129" s="4" t="n">
@@ -3663,12 +3663,12 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>53010003144104202606294024076281</t>
+          <t>53010003282126202606290211371154</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:56:37</t>
+          <t>2026-06-29 15:56:27</t>
         </is>
       </c>
       <c r="E130" s="4" t="n">
@@ -3688,12 +3688,12 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>53010003282126202606290211371154</t>
+          <t>53010003280188202606292664243214</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:56:27</t>
+          <t>2026-06-29 15:56:17</t>
         </is>
       </c>
       <c r="E131" s="4" t="n">
@@ -3713,12 +3713,12 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>53010003280188202606292664243214</t>
+          <t>53010003287162202606290064803261</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:56:17</t>
+          <t>2026-06-29 15:56:07</t>
         </is>
       </c>
       <c r="E132" s="4" t="n">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>53010003287162202606290064803261</t>
+          <t>53010003165248202606293511058812</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:56:07</t>
+          <t>2026-06-29 15:55:57</t>
         </is>
       </c>
       <c r="E133" s="4" t="n">
@@ -3763,12 +3763,12 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>53010003165248202606293511058812</t>
+          <t>53010003268115202606292201325098</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:55:57</t>
+          <t>2026-06-29 15:55:47</t>
         </is>
       </c>
       <c r="E134" s="4" t="n">
@@ -3788,12 +3788,12 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>53010003268115202606292201325098</t>
+          <t>53010003256037202606291433061585</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:55:47</t>
+          <t>2026-06-29 15:55:37</t>
         </is>
       </c>
       <c r="E135" s="4" t="n">
@@ -3813,12 +3813,12 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>53010003256037202606291433061585</t>
+          <t>53010003294048202606291918943726</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:55:37</t>
+          <t>2026-06-29 15:55:27</t>
         </is>
       </c>
       <c r="E136" s="4" t="n">
@@ -3838,12 +3838,12 @@
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>53010003294048202606291918943726</t>
+          <t>53010003151169202606292554837411</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:55:27</t>
+          <t>2026-06-29 15:55:16</t>
         </is>
       </c>
       <c r="E137" s="4" t="n">
@@ -3863,12 +3863,12 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>53010003151169202606292554837411</t>
+          <t>53010003156164202606293673134992</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:55:16</t>
+          <t>2026-06-29 15:55:04</t>
         </is>
       </c>
       <c r="E138" s="4" t="n">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>53010003156164202606293673134992</t>
+          <t>53010003285227202606291087429253</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:55:04</t>
+          <t>2026-06-29 15:54:52</t>
         </is>
       </c>
       <c r="E139" s="4" t="n">
@@ -3913,12 +3913,12 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>53010003285227202606291087429253</t>
+          <t>53010003166222202606290873937400</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:54:52</t>
+          <t>2026-06-29 15:54:41</t>
         </is>
       </c>
       <c r="E140" s="4" t="n">
@@ -3938,12 +3938,12 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>53010003166222202606290873937400</t>
+          <t>53010003251079202606292549047594</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:54:41</t>
+          <t>2026-06-29 15:54:28</t>
         </is>
       </c>
       <c r="E141" s="4" t="n">
@@ -3963,12 +3963,12 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>53010003251079202606292549047594</t>
+          <t>530100032552202606291979520460</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:54:28</t>
+          <t>2026-06-29 15:54:06</t>
         </is>
       </c>
       <c r="E142" s="4" t="n">
@@ -3988,12 +3988,12 @@
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>530100032552202606291979520460</t>
+          <t>53010003161222202606290281335611</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:54:06</t>
+          <t>2026-06-29 15:53:54</t>
         </is>
       </c>
       <c r="E143" s="4" t="n">
@@ -4013,12 +4013,12 @@
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>53010003161222202606290281335611</t>
+          <t>53010003264194202606293887561808</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:53:54</t>
+          <t>2026-06-29 15:53:42</t>
         </is>
       </c>
       <c r="E144" s="4" t="n">
@@ -4038,26 +4038,451 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>53010003264194202606293887561808</t>
+          <t>53010003289248202606294260685503</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 15:53:42</t>
+          <t>2026-06-29 15:53:26</t>
         </is>
       </c>
       <c r="E145" s="4" t="n">
         <v>150</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>53010003269124202606290952899173</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:52:57</t>
+        </is>
+      </c>
+      <c r="E146" s="4" t="n">
+        <v>130</v>
+      </c>
+    </row>
     <row r="147">
-      <c r="D147" s="5" t="inlineStr">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>53010003292095202606290921921229</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:52:41</t>
+        </is>
+      </c>
+      <c r="E147" s="4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>53010003145236202606290610210157</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:52:26</t>
+        </is>
+      </c>
+      <c r="E148" s="4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>活着viva</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>53010003289235202606293017409265</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:50:51</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>53010003268015202606290668138377</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:49:21</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>53010003249208202606293754387681</t>
+        </is>
+      </c>
+      <c r="D151" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:49:10</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>53010003144073202606291398143441</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:48:59</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>53010003278035202606293749686037</t>
+        </is>
+      </c>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:48:47</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>53010003144117202606292870825663</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:48:35</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>53010003288144202606293676122414</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:48:19</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>KK</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>53010003289039202606294083434878</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:48:05</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>稳住阵脚</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>53010003271109202606290197839852</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:39:09</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>稳住阵脚</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>53010003150059202606292040194179</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:38:56</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>稳住阵脚</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>53010003256068202606293579640115</t>
+        </is>
+      </c>
+      <c r="D159" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:38:43</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>稳住阵脚</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>53010003161138202606291744255426</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:38:15</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>稳住阵脚</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>53010003294210202606291623307683</t>
+        </is>
+      </c>
+      <c r="D161" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:36:55</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>18428341745</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>稳住阵脚</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>53010003144252202606290919882980</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-29 15:35:51</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="D164" s="5" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="E147" s="5" t="n">
-        <v>61351.79</v>
+      <c r="E164" s="5" t="n">
+        <v>58781.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>